<commit_message>
Rediseno visual completo con marca BitaLogs: dashboard, sidebar, PDF y logo
</commit_message>
<xml_diff>
--- a/BitaLogs_Export.xlsx
+++ b/BitaLogs_Export.xlsx
@@ -165,8 +165,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TablaAtenciones" displayName="TablaAtenciones" ref="A1:R24" headerRowCount="1">
-  <autoFilter ref="A1:R24"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TablaAtenciones" displayName="TablaAtenciones" ref="A1:R31" headerRowCount="1">
+  <autoFilter ref="A1:R31"/>
   <tableColumns count="18">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Fecha"/>
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R24"/>
+  <dimension ref="A1:R31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -502,9 +502,9 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="42" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
     <col width="24" customWidth="1" min="10" max="10"/>
     <col width="50" customWidth="1" min="11" max="11"/>
     <col width="50" customWidth="1" min="12" max="12"/>
@@ -610,61 +610,61 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>14:15</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Laboratorio</t>
+          <t>Emergencia</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Centrífuga</t>
+          <t>Maquina de Anestesia</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Drucker</t>
+          <t>DRE Medical</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Horizon 755VES</t>
+          <t>Transport 5000 Plus</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>160960AB219</t>
+          <t>AM803E18001004</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Preventivo</t>
+          <t>Revisión y Diagnóstico</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Se detectó durante mantenimiento preventivo que el equipo estaba descalibrado en cuanto el conteo de las RMP.</t>
+          <t>La maquina de anestesía no realiza "Flush" o purga de oxígeno.</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Se consultó manual de usuario para determinar como setear retardo al conteo en configuración avanzada del equipo. Posterior a la reprogramación se realizaron pruebas de funcionamiento para verificar el resultado deseado.</t>
+          <t>Se realizó la respectiva revisión de las válvula y mangueras del dispositivo siguiente el flujo de oxigeno para identificar obstrucciones. Se determinó que el mecanismo del cartucho de la válvula flush estaba atascado. El equipo queda operacional.</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
@@ -674,87 +674,95 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>Este retardo inicia el conteo el temporizador una vez el rotor alcanza las RPM colocadas (en este caso 3300 RPM) e inicia el conteo de las revoluciones en esa velocidad plena, asi la muestra recibe la fuerza completa durante todo el tiempo fijado, lo que influye directamente en la calidad de las muestras que impacta el estudio por ende los resultados vitales para el diagnóstico.</t>
+          <t>Se espera que este mecanismo de seguridad funcione adecuadamente ya que es vital en situaciones de emergencias donde se requiera aplicar un flujo rápido de oxigeno de forma bypass del flujómetro.</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>Equipo queda operacional.</t>
+          <t>Se recomienda sujetar con fajillas de velcro el equipo a su carrito de transporte para evitar la caída del dispositivo. Si el problema persiste se recomienda reemplazar el cartucho de la válvula flush PN: P04048.</t>
         </is>
       </c>
       <c r="P2" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q2" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R2" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Hospitalización B</t>
+          <t>Sala Cuna</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Cama Hospitalaria</t>
+          <t>Ventilador Mecánico Pediátrico</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Joson Care</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr"/>
-      <c r="I3" s="3" t="inlineStr"/>
+          <t>Drager</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Babylog-VN500</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>ASNB-0467</t>
+        </is>
+      </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
           <t>Preventivo</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>Durante la ronda diaria matutina, se detectó aue la cama de la habitación 25 de hospitalización B. No realizaba sus movimientos. Al estar desconectada se enchufó a la toma de pared y se procedió a pro ar sus respectivos movimientos descubriendo que de ifmra directa si realiza los movimientos. Se determinó que sis baterias están descargadas luego de hacer las pruebas correspondientes.</t>
-        </is>
-      </c>
+      <c r="K3" s="3" t="inlineStr"/>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>Se ingresó la solicitud al sistema interno del hospital para gestionar la entrega de las baterias de la bodega de mantenimiento. Una vez entregadas se probaron los voltajes y estos estaban muy bajos. (9.77 v y 11.9 v) respectivamente. Por lo que requieran un tiempo de carga.</t>
+          <t>Se realizó mantenimiento preventivo según el manual de servicio que provee el fabricante. El Dispositivo realizó todas las pruebas de autotest previo a la instalación del circuito de paciente y aprobó cada una de las evaluaciones.</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>Parcial</t>
-        </is>
-      </c>
-      <c r="N3" s="3" t="inlineStr"/>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>Al dar mantenimiento preventivo al babylog-vn500 no solo prolongamos la vida útil del dispositivo, también contribuye a las terapias realizadas a los neonatos en necesidad de una respiración asistida.</t>
+        </is>
+      </c>
       <c r="O3" s="3" t="inlineStr"/>
       <c r="P3" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q3" s="3" t="n">
         <v>2</v>
-      </c>
-      <c r="Q3" s="3" t="n">
-        <v>4</v>
       </c>
       <c r="R3" s="3" t="n">
         <v>60</v>
@@ -762,80 +770,80 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>69</v>
+        <v>83</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>10:45</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Laboratorio</t>
+          <t>Sala Cuna</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Set de Diagnóstico Pediátrico</t>
+          <t>Cascada F. P.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Welch Allyn</t>
+          <t>Fisher Paykel</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Fibra óptica</t>
+          <t>MR-850JSU</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>05681</t>
+          <t>50222002916</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Correctivo</t>
+          <t>Revisión y Diagnóstico</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>La luz se apaga y se enciende esporádicamente</t>
+          <t>Equipo se inicia y presenta en su pantalla de display error #21, contrario a lo reportado por el personal (error#19).</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Se observo el laringoscopio del set de diagnóstico y se determinó un falso contacto posterior a varias priebas de funcionamiento. Se estaño la bombilla para entender el contacto. Se recomienda el reemplazo de ambas bombillas.</t>
+          <t>Se realizó la respectiva revisión, el display mostraba error 21 y emitía una alarma. Se consultó el manual de servicio que provee el fabricante donde sugiere iante este error el reemplazo de la PCB. Al analizar internamente el equipo se ven signos indicadores de deterioro interno por lo que el equipo no es operacional y se le da de baja.</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>Parcial</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>Al quedar funcional el laringiscopio es vital para un intubación correcta. Sumamente importante en el area de emergencias en la instancia que el paciente requiera apoyo para cinolir la función respiratoria por medio de ventilación mecánica</t>
+          <t>El área de sala cuna solo queda con 3 de las 5 cascadas de oxígeno asignadas al área. Lo que en su momento limitará la disponibilidad de las mismas.</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>El equipo queda funcional y operacional. Se recomienda el reemplazo de ambas bombillas PN: HPX060 y tener en stock. (2)</t>
+          <t>Es recomendable la adquisición de un equipo nuevo por sobre el el reemplazo de la PCB ya que su precio se encenetra en rangos similares.</t>
         </is>
       </c>
       <c r="P4" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q4" s="2" t="n">
         <v>2</v>
@@ -846,213 +854,229 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
-        <v>56</v>
+        <v>82</v>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>11:45</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio</t>
+          <t>Sala Cuna</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Centrífuga</t>
+          <t>Incubadora Neonatal</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>LWS</t>
+          <t>General Electric</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>V24T</t>
+          <t>Giraffe Omnibed</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>14090366</t>
+          <t>TABZ-7009</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>Preventivo</t>
-        </is>
-      </c>
-      <c r="K5" s="3" t="inlineStr"/>
+          <t>Revisión y Diagnóstico</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>Equipo emite sonidos molestos intermitentes que parece provienen del motor.</t>
+        </is>
+      </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>Se realizó mantenimiento preventivo de acuerdo al manual del fabricante. se hicieron pruebas de funcionamiento, limpieza exterior e interior de los portatubos y rotor. Se tomó nota de las RPM (promedio 3308.2  RPM) para llevar registro ya que los laboratorios son certificados bajo la IS09001 2015. Se remendó sticker de botonera start/stop ya que presentaba desgaste por uso.</t>
+          <t>Se realizó la revisión y el sistema presenta una falla en el motor del ventilador lo que emite fallos y sonidos intermitentes, Se requiere el reemplazo a corto plazo del sensor óptico, bushing, propela, ya que puede quedar inoperable.</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>Al realizar los mantenimientos correctivos correspondientes en la periodicidad descrita por el fabricante se mantiene la vida útil del dispositivo y garantiza el buen funcionamiento, crucial en este caso para mantener la certificación del laboratorio, lo que proyecta seguridad en los resultados de los procedimientos realizados.</t>
+          <t>Se espera la adquisición de los repuestos indicados para su instalación a corto plazo ya que el dispositivo podría quedar completamente inoperable si se permite que el deterioro avance.</t>
         </is>
       </c>
       <c r="O5" s="3" t="inlineStr">
         <is>
-          <t>Equipo queda funcional y operando.</t>
+          <t>Se recomienda el reemplazo del motor PN: 6600-1057-600; fan hub PN: 6600-1440-500; fan seal 6600-1557-500; optical sensor holder PN: 6600-1435-500; optical gasket PN: 6600_1437500.</t>
         </is>
       </c>
       <c r="P5" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q5" s="3" t="n">
         <v>2</v>
       </c>
       <c r="R5" s="3" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Laboratorio</t>
+          <t>Quirófano 2</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Incubadora de Laboratorio </t>
+          <t>Máquina de Anestesia</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Lab Line</t>
+          <t>General Electric</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>Aespire</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>04-081332</t>
+          <t>AMXS00841</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Preventivo</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr"/>
+          <t>Revisión y Diagnóstico</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>El anestesiólogo encargado reporta que el equipo presenta una alarma de baja saturación de oxigeno al 19% cuando idealmente debe de estar en 21%.</t>
+        </is>
+      </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Se realizó mantenimiento preventivo mediante la limpieza y desinfección profunda, la calibración de temperatura y sensores, y la inspección de componentes mecánicos y filtros</t>
+          <t>Se realizó la revisión del equipo y se identifico que las celdas de oxigeno estaban dañadas tras la realización de las calibraciones de oxigeno sugeridas por fabricante al 21% y al 100% el equipo no pasó ambas lo que indica que la celda de oxigeno necesita ser reemplazada. Se pasó reporte de esto a compras para gestionar la adquisición de 3 celdas de oxigeno ya que semanas anteriores en el 19 de julio otro equipo tuvo el mismo problema y se encuentra de baja por lo mismo.</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>se espera que continue a crear y mantener un ambiente controlado óptimo para cultivar microorganismos, mantener cultivos celulares y almacenar muestras biológicas.</t>
-        </is>
-      </c>
-      <c r="O6" s="2" t="inlineStr"/>
+          <t>Se espera que con el reporte formalizado firmado por el encargado de área compras autorice la adquisición de 3 celdas nuevas 2 par reemplazo y 1 para tener en stock ya que existen 5 equipo de misma marca y modelo contando los 2 que están temporalmente de baja.</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>Se recomienda el reemplazo de las dos celdas a corto plazo en los próximos días.</t>
+        </is>
+      </c>
       <c r="P6" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q6" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R6" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Laboratorio</t>
+          <t>Quirófano 4</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Agitador Rotador</t>
+          <t>Unidad de Electrocirugía</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Lab Rotator</t>
+          <t>Valleylab</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>L-RT28</t>
+          <t>Force FX-C</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>0809391</t>
+          <t>F8D60776A</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>Preventivo</t>
-        </is>
-      </c>
-      <c r="K7" s="3" t="inlineStr"/>
+          <t>Revisión y Diagnóstico</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>Personal de quirófano 4 reporta que no se acciona el lápiz. Una vez en la mesa de trabajo de biómedica de determinó que no se accionaba la ESU  ya que no estaba bien cerrado el circuito de paciente debido a mal manejo del personal. se detectó que se le estaba dando múltiples usos a la placa de retorno desechable y esta estaba comprometida, por ll que al reemplazar esta y el lápiz, la ESU realizaba y pasaba su autotest y se permitía realizar cortes y coagulación monopolar.</t>
+        </is>
+      </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>Se realizó mantenimiento preventivo. de acuerdo al manual de usuario. Limpieza exterior con alcohol isopropílico al 80% y se revisaron el funcionamiento de sus partes mecánicas.</t>
+          <t>Se reemplazo la placa de retorno o que cerró el circuito y funciona a normalmente.</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
@@ -1062,73 +1086,81 @@
       </c>
       <c r="N7" s="3" t="inlineStr">
         <is>
-          <t>Se espera el correcto funcionamiento para que mantenga su función de mezclar líquidos en los tubos mediante sus movimientos circulares giratorios.</t>
-        </is>
-      </c>
-      <c r="O7" s="3" t="inlineStr"/>
+          <t>Al utilizar el equipo debidamente se mantiene la seguridad eléctrica tanto para el paciente como para el usuario lo que limita la posibilidad de quemaduras o efetos adversos de la ESU al tener el circuito de retorno activo y funcional.</t>
+        </is>
+      </c>
+      <c r="O7" s="3" t="inlineStr">
+        <is>
+          <t>Se recomienda no darles múltiples uso a las placas de retorno de paciente.</t>
+        </is>
+      </c>
       <c r="P7" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q7" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R7" s="3" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>14:45</t>
+          <t>10:45</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Laboratorio</t>
+          <t>HDV La Lima</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Centrífuga</t>
+          <t>Camilla de parada</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Unico</t>
+          <t>Nitrocare</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>C8724</t>
+          <t>NTCR SD01</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>1408147</t>
+          <t>01-0558</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Preventivo</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr"/>
+          <t>Correctivo</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>El amortiguador hidráulico tenia una pieza rota lo que no permitía la tensión de sus cables para hacer los movimientos de espalda y Trendelenburg controlados.</t>
+        </is>
+      </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Se realizó mantenimiento preventivo. Se limpió profundamente su exterior, rotor, compuerta, y el set de 24 portatubos. Se realizaron pruebas de RPM con fototacómetro para asegurar que cumplía con el estándar de la certificación para una centrifuga de orina (2500 rpm). Se desvastó la parte interna de los portatubos para asegurar el ingreso y salida de los tubos sin dificultad ya que se identificó que la fuerza centrípeta ocasionaba la defomación del plástico interno.</t>
+          <t>Se remplazaron los componentes rotos del amortiguador y se hicieron varias pruebas de funcionamiento. el equipo las paso todas al hacer los movimientos controlados por la palanca hidráulica.</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
@@ -1138,27 +1170,27 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>Al realizar los mantenimientos correctivos correspondientes en la periodicidad descrita por el fabricante se mantiene la vida útil del dispositivo y garantiza el buen funcionamiento, crucial en este caso para mantener la certificación del laboratorio, lo que proyecta seguridad en los resultados de los procedimientos realizados.</t>
+          <t>Se espera que la camilla realice los movimientos adecuados incluyendo Trendelenburg para mejorar el retorno venoso al corazón de los pacientes que lo requieran.</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr"/>
       <c r="P8" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q8" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R8" s="2" t="n">
-        <v>15</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -1178,22 +1210,22 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Micro Centrífuga</t>
+          <t>Centrífuga</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Unico</t>
+          <t>Drucker</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>CMH30</t>
+          <t>Horizon 755VES</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>0908466</t>
+          <t>160960AB219</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
@@ -1201,10 +1233,14 @@
           <t>Preventivo</t>
         </is>
       </c>
-      <c r="K9" s="3" t="inlineStr"/>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>Se detectó durante mantenimiento preventivo que el equipo estaba descalibrado en cuanto el conteo de las RMP.</t>
+        </is>
+      </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>Se realizó mantenimiento preventivo del equipo. Asegurando funcionamiento pre-post mantenimiento. Se midieron las RPM con un fototacómetro. se obtuvo el promedio de 9591.4 RPM.</t>
+          <t>Se consultó manual de usuario para determinar como setear retardo al conteo en configuración avanzada del equipo. Posterior a la reprogramación se realizaron pruebas de funcionamiento para verificar el resultado deseado.</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr">
@@ -1214,15 +1250,19 @@
       </c>
       <c r="N9" s="3" t="inlineStr">
         <is>
-          <t>Se espera siga operando de adecuada contribuyendo al estudio de volúmenes reducidos para el análisis de fluidos biológicos.</t>
-        </is>
-      </c>
-      <c r="O9" s="3" t="inlineStr"/>
+          <t>Este retardo inicia el conteo el temporizador una vez el rotor alcanza las RPM colocadas (en este caso 3300 RPM) e inicia el conteo de las revoluciones en esa velocidad plena, asi la muestra recibe la fuerza completa durante todo el tiempo fijado, lo que influye directamente en la calidad de las muestras que impacta el estudio por ende los resultados vitales para el diagnóstico.</t>
+        </is>
+      </c>
+      <c r="O9" s="3" t="inlineStr">
+        <is>
+          <t>Equipo queda operacional.</t>
+        </is>
+      </c>
       <c r="P9" s="3" t="n">
         <v>2</v>
       </c>
       <c r="Q9" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R9" s="3" t="n">
         <v>15</v>
@@ -1230,48 +1270,40 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>13:45</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Laboratorio</t>
+          <t>Hospitalización B</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Centrífuga</t>
+          <t>Cama Hospitalaria</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Humax</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>5K</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>01-05505</t>
-        </is>
-      </c>
+          <t>Joson Care</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr">
         <is>
           <t>Preventivo</t>
@@ -1279,52 +1311,48 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Tubos se atascaban en el portatubos</t>
+          <t>Durante la ronda diaria matutina, se detectó aue la cama de la habitación 25 de hospitalización B. No realizaba sus movimientos. Al estar desconectada se enchufó a la toma de pared y se procedió a pro ar sus respectivos movimientos descubriendo que de ifmra directa si realiza los movimientos. Se determinó que sis baterias están descargadas luego de hacer las pruebas correspondientes.</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Se realizó mantenimiento preventivo. Se limpió profundamente su exterior, rotor, compuerta, y el set de 24 portatubos. Se realizaron pruebas de RPM con fototacómetro para asegurar que cumplía con el estándar de la certificación para una centrifuga de orina (2500 rpm). Se desvastó la parte interna de los portatubos para asegurar el ingreso y salida de los tubos sin dificultad ya que se identificó que la fuerza centrípeta ocasionaba la defomación del plástico interno.</t>
+          <t>Se ingresó la solicitud al sistema interno del hospital para gestionar la entrega de las baterias de la bodega de mantenimiento. Una vez entregadas se probaron los voltajes y estos estaban muy bajos. (9.77 v y 11.9 v) respectivamente. Por lo que requieran un tiempo de carga.</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="N10" s="2" t="inlineStr">
-        <is>
-          <t>Se espera siga cumpliendo su función de generar suspensión de cristales y estratificación de fluidos.</t>
-        </is>
-      </c>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr"/>
       <c r="O10" s="2" t="inlineStr"/>
       <c r="P10" s="2" t="n">
         <v>2</v>
       </c>
       <c r="Q10" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R10" s="2" t="n">
-        <v>15</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -1334,46 +1362,54 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Baño María</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr"/>
+          <t>Set de Diagnóstico Pediátrico</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Welch Allyn</t>
+        </is>
+      </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>Precisterm</t>
+          <t>Fibra óptica</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>05-0366</t>
+          <t>05681</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>Preventivo</t>
+          <t>Correctivo</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>Biofilm en la superficie del agua</t>
+          <t>La luz se apaga y se enciende esporádicamente</t>
         </is>
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>Se realizo mantenimiento preventivo del dispositivo. Una limpieza profunda del recipiente, su rejilla, y su resistencia. Se realizo prueba de funcionamiento con un termómetro y se obtuvo el resultado esperado.</t>
+          <t>Se observo el laringoscopio del set de diagnóstico y se determinó un falso contacto posterior a varias priebas de funcionamiento. Se estaño la bombilla para entender el contacto. Se recomienda el reemplazo de ambas bombillas.</t>
         </is>
       </c>
       <c r="M11" s="3" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="N11" s="3" t="inlineStr">
         <is>
-          <t>Se espera contuinue funcionando adecuadamente en la asistencia de los cultivos y temperización de muestras-.</t>
-        </is>
-      </c>
-      <c r="O11" s="3" t="inlineStr"/>
+          <t>Al quedar funcional el laringiscopio es vital para un intubación correcta. Sumamente importante en el area de emergencias en la instancia que el paciente requiera apoyo para cinolir la función respiratoria por medio de ventilación mecánica</t>
+        </is>
+      </c>
+      <c r="O11" s="3" t="inlineStr">
+        <is>
+          <t>El equipo queda funcional y operacional. Se recomienda el reemplazo de ambas bombillas PN: HPX060 y tener en stock. (2)</t>
+        </is>
+      </c>
       <c r="P11" s="3" t="n">
         <v>2</v>
       </c>
@@ -1386,21 +1422,21 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>11:45</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1410,18 +1446,22 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Microscopio</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr"/>
+          <t>Centrífuga</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>LWS</t>
+        </is>
+      </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>8D06-705</t>
+          <t>V24T</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>CX21FS1</t>
+          <t>14090366</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1432,7 +1472,7 @@
       <c r="K12" s="2" t="inlineStr"/>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Se realizó mantenimiento preventivo al equipo según plan de mantenimiento de la empresa. Se limpiaron a  profundidad sus componentes, la base, el foco, el brazo revólver, objetivo, tubo etc.</t>
+          <t>Se realizó mantenimiento preventivo de acuerdo al manual del fabricante. se hicieron pruebas de funcionamiento, limpieza exterior e interior de los portatubos y rotor. Se tomó nota de las RPM (promedio 3308.2  RPM) para llevar registro ya que los laboratorios son certificados bajo la IS09001 2015. Se remendó sticker de botonera start/stop ya que presentaba desgaste por uso.</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
@@ -1442,10 +1482,14 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>Se espera que con la remoción de la suciedad en el foco pueda ayudar a realizar los estudios correspondientes.</t>
-        </is>
-      </c>
-      <c r="O12" s="2" t="inlineStr"/>
+          <t>Al realizar los mantenimientos correctivos correspondientes en la periodicidad descrita por el fabricante se mantiene la vida útil del dispositivo y garantiza el buen funcionamiento, crucial en este caso para mantener la certificación del laboratorio, lo que proyecta seguridad en los resultados de los procedimientos realizados.</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>Equipo queda funcional y operando.</t>
+        </is>
+      </c>
       <c r="P12" s="2" t="n">
         <v>2</v>
       </c>
@@ -1458,7 +1502,7 @@
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
-        <v>57</v>
+        <v>76</v>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
@@ -1467,12 +1511,12 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>11:15</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>15:45</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -1482,22 +1526,22 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>CentrÍfuga</t>
+          <t xml:space="preserve">Incubadora de Laboratorio </t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Drucker</t>
+          <t>Lab Line</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>Horizon 755VES</t>
+          <t>150</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>160960AB219</t>
+          <t>04-081332</t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr">
@@ -1508,7 +1552,7 @@
       <c r="K13" s="3" t="inlineStr"/>
       <c r="L13" s="3" t="inlineStr">
         <is>
-          <t>Se realzó mantenimiento preventivo según el manual del fabricante. Se ajustaron las patas de goma ante leve movimiento. Se realizó una limpieza exterior del equipo y un lavado profundo de los portatubos, se procedió a a realizar las pruebas de RPM con el fototacómetro para determinar si esta en rango tolerable. Se remendaron las botoneras on/ off. equipo queda funcional y operativo.</t>
+          <t>Se realizó mantenimiento preventivo mediante la limpieza y desinfección profunda, la calibración de temperatura y sensores, y la inspección de componentes mecánicos y filtros</t>
         </is>
       </c>
       <c r="M13" s="3" t="inlineStr">
@@ -1518,7 +1562,7 @@
       </c>
       <c r="N13" s="3" t="inlineStr">
         <is>
-          <t>Al realizar los mantenimientos preventivos correspondientes aseguramos el buen funcionamiento del equipo extendemos su vida util, y certificamos los resultados de laboratorio.</t>
+          <t>se espera que continue a crear y mantener un ambiente controlado óptimo para cultivar microorganismos, mantener cultivos celulares y almacenar muestras biológicas.</t>
         </is>
       </c>
       <c r="O13" s="3" t="inlineStr"/>
@@ -1534,46 +1578,46 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>15:15</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Hospitalización A</t>
+          <t>Laboratorio</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Monitor Fetal</t>
+          <t>Agitador Rotador</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Edan</t>
+          <t>Lab Rotator</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>L-RT28</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>M-19303227002</t>
+          <t>0809391</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1581,36 +1625,28 @@
           <t>Preventivo</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>Durante el recorrido matutino diario se observó en bodega de Hospitalización a el monitor Fetal Edan M2. Este con evidencia clara de desgaste en sus transductores de Ultrasonido y TOCO. Anteriormente se habían remendado temporalmente pero el desgaste es evidente. Se documenta que el monitor detal de la misma marca y modelo ubicado en emergencias presenta los mismos indicios lo cual los vuelve casi inoperables y está en riesgo de mal funcionamiento de forma inminente.</t>
-        </is>
-      </c>
+      <c r="K14" s="2" t="inlineStr"/>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>Se realizaron reportes técnicos y cotizaciónes para el reemplazo total de ambos set de transductores (US y TOCO) para los monitores fetales de Hospitalización A y Emergencias ya que se recomienda reemplazar los actuales a corto plazo con prontitud.</t>
+          <t>Se realizó mantenimiento preventivo. de acuerdo al manual de usuario. Limpieza exterior con alcohol isopropílico al 80% y se revisaron el funcionamiento de sus partes mecánicas.</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>Parcial</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>Se espera que la adquisición de los nuevos transductores ayude a garantizar la fiabilidad de los datos obtenidos en cada monitoreo fetal realizado con estos equipos.</t>
-        </is>
-      </c>
-      <c r="O14" s="2" t="inlineStr">
-        <is>
-          <t>Los equipos actualmente se encuentran operacionales pero ante este tipo de desgaste el manual de servicio recomienda el reemplazo de los transductores para evitar errores en los estudios.</t>
-        </is>
-      </c>
+          <t>Se espera el correcto funcionamiento para que mantenga su función de mezclar líquidos en los tubos mediante sus movimientos circulares giratorios.</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr"/>
       <c r="P14" s="2" t="n">
         <v>2</v>
       </c>
       <c r="Q14" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R14" s="2" t="n">
         <v>15</v>
@@ -1618,57 +1654,57 @@
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>10:15</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>14:45</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Emergencia</t>
+          <t>Laboratorio</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Balanzas Pediátricas y de adulto</t>
+          <t>Centrífuga</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Detecto</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="inlineStr"/>
+          <t>Unico</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>C8724</t>
+        </is>
+      </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>127566</t>
+          <t>1408147</t>
         </is>
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>Correctivo</t>
-        </is>
-      </c>
-      <c r="K15" s="3" t="inlineStr">
-        <is>
-          <t>Las balanzas pediátricas de emergencia se encontraron descalibradas en el recorrido matutino diario de las áreas, esto ya que fueron movidas y se descalibró el contrapeso.</t>
-        </is>
-      </c>
+          <t>Preventivo</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr"/>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>Se ajusto el tornillo del contrapeso cuidadosamente girando levemente a favor de las manecillas del reloj, soltando el indicador asegurando encontrara su punto de balance enmedio de la guia de peso.</t>
+          <t>Se realizó mantenimiento preventivo. Se limpió profundamente su exterior, rotor, compuerta, y el set de 24 portatubos. Se realizaron pruebas de RPM con fototacómetro para asegurar que cumplía con el estándar de la certificación para una centrifuga de orina (2500 rpm). Se desvastó la parte interna de los portatubos para asegurar el ingreso y salida de los tubos sin dificultad ya que se identificó que la fuerza centrípeta ocasionaba la defomación del plástico interno.</t>
         </is>
       </c>
       <c r="M15" s="3" t="inlineStr">
@@ -1678,7 +1714,7 @@
       </c>
       <c r="N15" s="3" t="inlineStr">
         <is>
-          <t>Las personas ingresadas por medio de emergencias tendrán lecturas mas certeras de su peso lo cual es de mucha importancia para el personal de la salud al momento de suministrar medicamentos o determinar diagnósticos.</t>
+          <t>Al realizar los mantenimientos correctivos correspondientes en la periodicidad descrita por el fabricante se mantiene la vida útil del dispositivo y garantiza el buen funcionamiento, crucial en este caso para mantener la certificación del laboratorio, lo que proyecta seguridad en los resultados de los procedimientos realizados.</t>
         </is>
       </c>
       <c r="O15" s="3" t="inlineStr"/>
@@ -1686,7 +1722,7 @@
         <v>2</v>
       </c>
       <c r="Q15" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R15" s="3" t="n">
         <v>15</v>
@@ -1694,21 +1730,21 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>58</v>
+        <v>73</v>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>14:15</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1718,81 +1754,73 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Centrífuga</t>
+          <t>Micro Centrífuga</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Drucker</t>
+          <t>Unico</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>755 VES</t>
+          <t>CMH30</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>160960AB218</t>
+          <t>0908466</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Revisión y Diagnóstico</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>Laboratorio solicitó revisión y diagnóstico de la centrífuga Drucker Horizon 755 VES. ya que esta no iniciaba y según relato del Dr. encargado del área (Rubén Vallecillo) emitió humo antes de dejar de funcionar. Se observó internamente una falla crítica en la tarjeta electrónica principal. Múltiples de los integrados de la placa presentan carbonización lo que compromete el funcionamiento del equipo.</t>
-        </is>
-      </c>
+          <t>Preventivo</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr"/>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">La sustitución de los componentes microsoldados no resulta viable, ya que se corre el riesgo de comprometer otros componentes en el proceso. El equipo queda fuera de servicio hasta el reemplazo de la tarjeta principal. Se adjuntará cotización de la parte PN-7717041 (Placa electrónica principal centrífuga Drucker  Horizon 755 VES) al reporte entregado a mantenimiento para agilizar la respectiva compra / adquisición. Mientras tanto, el equipo queda de baja. Se recomienda una UPS de 1.5 KVA para mitigar el impacto de los picos de voltaje ya que la laca es inverter y susceptible a esto. </t>
+          <t>Se realizó mantenimiento preventivo del equipo. Asegurando funcionamiento pre-post mantenimiento. Se midieron las RPM con un fototacómetro. se obtuvo el promedio de 9591.4 RPM.</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>Se espera que por medio del reporte entregado a mantenimiento se pueda adquirir la placa para el reemplazo de la tarjeta su reparo, pruebas de funcionamiento y calibración para devolverlo en estado funcional y operable a su área (laboratorio)</t>
-        </is>
-      </c>
-      <c r="O16" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">El equipo queda fuera de servicio. El problema será recurrente ante la falta de un UPS para proteger el equipo de picos de voltaje. </t>
-        </is>
-      </c>
+          <t>Se espera siga operando de adecuada contribuyendo al estudio de volúmenes reducidos para el análisis de fluidos biológicos.</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr"/>
       <c r="P16" s="2" t="n">
         <v>2</v>
       </c>
       <c r="Q16" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R16" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>13:45</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
@@ -1802,25 +1830,37 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Incubadora de Laboratorio</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr"/>
-      <c r="H17" s="3" t="inlineStr"/>
-      <c r="I17" s="3" t="inlineStr"/>
+          <t>Centrífuga</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Humax</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>5K</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>01-05505</t>
+        </is>
+      </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>Correctivo</t>
+          <t>Preventivo</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>Se solicitò asistencia de parte de mantenimiento en el arèa de laboratorio ya qye su incubadora proncipal tiene emn mal estado la puerta, lo que pone en riesgo los cultivos dentro del mismo. Al examinar el equipo estaba unicamente cerrado con cinta adhesiva ya que el mecanismo de cierre se descompuso. Se desmontó la puerta para ver el mecanismo y se encuentra roto</t>
+          <t>Tubos se atascaban en el portatubos</t>
         </is>
       </c>
       <c r="L17" s="3" t="inlineStr">
         <is>
-          <t>Se soldó el seguro interno (Abrir/cerrar) de la puerta sujeto a la maniblea y se reemplazaron los tornillos por unos de mayor alcance para asegurar que no se salgan se sus ubicaciones.</t>
+          <t>Se realizó mantenimiento preventivo. Se limpió profundamente su exterior, rotor, compuerta, y el set de 24 portatubos. Se realizaron pruebas de RPM con fototacómetro para asegurar que cumplía con el estándar de la certificación para una centrifuga de orina (2500 rpm). Se desvastó la parte interna de los portatubos para asegurar el ingreso y salida de los tubos sin dificultad ya que se identificó que la fuerza centrípeta ocasionaba la defomación del plástico interno.</t>
         </is>
       </c>
       <c r="M17" s="3" t="inlineStr">
@@ -1830,133 +1870,145 @@
       </c>
       <c r="N17" s="3" t="inlineStr">
         <is>
-          <t>Se esper que el personal siga las recomendaciones de no ejercer fuerza excesiva al abrir y cerrar ya que el mecanismo puede volver a quebrarse.</t>
+          <t>Se espera siga cumpliendo su función de generar suspensión de cristales y estratificación de fluidos.</t>
         </is>
       </c>
       <c r="O17" s="3" t="inlineStr"/>
       <c r="P17" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q17" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="R17" s="3" t="n">
-        <v>120</v>
+        <v>15</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>13:15</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>UCIN</t>
+          <t>Laboratorio</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Incubadora Neonatal</t>
+          <t>Baño María</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr"/>
-      <c r="H18" s="2" t="inlineStr"/>
-      <c r="I18" s="2" t="inlineStr"/>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Precisterm</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>05-0366</t>
+        </is>
+      </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Correctivo</t>
+          <t>Preventivo</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>La Incubadora noenatal GE giraffe Omnibed presenta probelmas perisistentes en su motor. Anteriormente se realizó antenimimento correctivo de las balineras. Actuakmente se solicita ayuda por "Sonidos fuertes" provinientes del dispositivo.</t>
+          <t>Biofilm en la superficie del agua</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>Posterior al analisis de los componentes internos una ves se remueve su carcaza, se determino que piezas especificas como el motor, sensor optico, plasticos de acoplo requieren ser reemplazados,</t>
+          <t>Se realizo mantenimiento preventivo del dispositivo. Una limpieza profunda del recipiente, su rejilla, y su resistencia. Se realizo prueba de funcionamiento con un termómetro y se obtuvo el resultado esperado.</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>Se esperan solicitudoes de atencion por el sonido intermitente que recurre en el motor. Se solci´to la compra de respuestos para atender el problema de raiz.</t>
-        </is>
-      </c>
-      <c r="O18" s="2" t="inlineStr">
-        <is>
-          <t>queda operacional con los ruidos intermitentes.y se recomienda el reemplazo de las piezas entregadas a gerente de mantenimineto con sus repspectiva cotización para compra.</t>
-        </is>
-      </c>
+          <t>Se espera contuinue funcionando adecuadamente en la asistencia de los cultivos y temperización de muestras-.</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr"/>
       <c r="P18" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q18" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="R18" s="2" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>9:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>09:30</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr"/>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Laboratorio</t>
+        </is>
+      </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Tomgrafo</t>
+          <t>Microscopio</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr"/>
-      <c r="H19" s="3" t="inlineStr"/>
-      <c r="I19" s="3" t="inlineStr"/>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>8D06-705</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>CX21FS1</t>
+        </is>
+      </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>Correctivo</t>
-        </is>
-      </c>
-      <c r="K19" s="3" t="inlineStr">
-        <is>
-          <t>Se hizó al la observación al peronal de Biotec que el inicializar el tomógrafo CT-300 Philips en cada báarido aparecia un mensaje de error emitido por el software. Tras una revisión de determino que el disco duro estaba próximo a alacanzar su capacidad máximo la que pone en riesgo la "Raw data" ante corrupciones por sobre carga de información, de igual forma se expuso que el equipo se mantiene encendido 24/7.</t>
-        </is>
-      </c>
+          <t>Preventivo</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr"/>
       <c r="L19" s="3" t="inlineStr">
         <is>
-          <t>Se recomendó al personal depurar de estudios muy antiguos el disco duro del ordenador. Ya que la sobrecarga del mismo presenta el riesgo de coorromper la raw data de estudios recientes. El sistema muestra advenrtencias por esta situación, pero ningun error fatal de sistema si se siguen las indicaciones. De igual forma se recomendó apagar el ordenador un par de minutos mínimo 1 vezpor semana.</t>
+          <t>Se realizó mantenimiento preventivo al equipo según plan de mantenimiento de la empresa. Se limpiaron a  profundidad sus componentes, la base, el foco, el brazo revólver, objetivo, tubo etc.</t>
         </is>
       </c>
       <c r="M19" s="3" t="inlineStr">
@@ -1966,65 +2018,73 @@
       </c>
       <c r="N19" s="3" t="inlineStr">
         <is>
-          <t>Se espera que el persnal siga las recomiendaciones e indicaciones del personal técncico para evitar la sobre carga del disco duro, ya que esto pone en riesgo la calidad de los estudios y la información adquirida para diagnóstico.</t>
+          <t>Se espera que con la remoción de la suciedad en el foco pueda ayudar a realizar los estudios correspondientes.</t>
         </is>
       </c>
       <c r="O19" s="3" t="inlineStr"/>
       <c r="P19" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q19" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R19" s="3" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>11:15</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Hospitalización A</t>
+          <t>Laboratorio</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Termómetro de oído</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr"/>
-      <c r="H20" s="2" t="inlineStr"/>
-      <c r="I20" s="2" t="inlineStr"/>
+          <t>CentrÍfuga</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Drucker</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Horizon 755VES</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>160960AB219</t>
+        </is>
+      </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>Correctivo</t>
-        </is>
-      </c>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
-          <t>En una visita al área, personal de enfermería de Hospitalización B expusó que los termometro de oido portátil del MSV Welch Allyn LXI 45NTO Tenia sus baterías descargadas. Se canbiaron las mismas por unas cagadas y el termómetro no operó. Al ver sus componentes internos, se observía que en su placa un falso contacto con la bandeja de batería por el desgaste de la constante driccion entre la bandeja y la placa.</t>
-        </is>
-      </c>
+          <t>Preventivo</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr"/>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>Posterior a la vista intenra de la tarjeta del equipo se realizaron varias pruebas de utilizando aluminio como medio de conduccion entre la placa y la bandeja de bateria. Estas pruebas no dieron resultado ya que el plastico de cierre ya estaba sumamente desgastado lo que no permitia que cerrara bien. Como existe repuesto total del dispositovo se optó por remplazarlo en su totalidad. y queda funcional y operando.</t>
+          <t>Se realzó mantenimiento preventivo según el manual del fabricante. Se ajustaron las patas de goma ante leve movimiento. Se realizó una limpieza exterior del equipo y un lavado profundo de los portatubos, se procedió a a realizar las pruebas de RPM con el fototacómetro para determinar si esta en rango tolerable. Se remendaron las botoneras on/ off. equipo queda funcional y operativo.</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
@@ -2034,65 +2094,77 @@
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>Al ser equipo de atiguedad dentro del área, se sepera que termomentro adjunto al MSV de su vida util para reemplazar el monitor en su totalidad.</t>
+          <t>Al realizar los mantenimientos preventivos correspondientes aseguramos el buen funcionamiento del equipo extendemos su vida util, y certificamos los resultados de laboratorio.</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr"/>
       <c r="P20" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q20" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R20" s="2" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>09:15</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Hospitalización B</t>
+          <t>Hospitalización A</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Monitor de Signos vitales</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr"/>
-      <c r="H21" s="3" t="inlineStr"/>
-      <c r="I21" s="3" t="inlineStr"/>
+          <t>Monitor Fetal</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Edan</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>M-19303227002</t>
+        </is>
+      </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
-          <t>Correctivo</t>
+          <t>Preventivo</t>
         </is>
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>Se solicitó apoyo de por medio de un aorden de mantenimiento para inspeccionar el MSV Mindray VS-900 C de Hospitalización A, ya que este no sensa temperatura y la sonda de temperatura parece estar en buen estado. Se inpseccionó mas a detalle internamente y se determinó que el "sheath" o funda donde se coloca la sonda de temp. esta rota. y la guia de la misma no hace contacto con el sensor por medio de una botornera.</t>
+          <t>Durante el recorrido matutino diario se observó en bodega de Hospitalización a el monitor Fetal Edan M2. Este con evidencia clara de desgaste en sus transductores de Ultrasonido y TOCO. Anteriormente se habían remendado temporalmente pero el desgaste es evidente. Se documenta que el monitor detal de la misma marca y modelo ubicado en emergencias presenta los mismos indicios lo cual los vuelve casi inoperables y está en riesgo de mal funcionamiento de forma inminente.</t>
         </is>
       </c>
       <c r="L21" s="3" t="inlineStr">
         <is>
-          <t>Se implemento el ingenio para elaborar una extensión a la funda que hace contacto con el sensor ya que este fue el que se quebró e impide el funcionamiento del módulo de temperatura del MSV. Se lógro proporcionar esta solución temporal y el equipo queda funacional tras varias pruebas.</t>
+          <t>Se realizaron reportes técnicos y cotizaciónes para el reemplazo total de ambos set de transductores (US y TOCO) para los monitores fetales de Hospitalización A y Emergencias ya que se recomienda reemplazar los actuales a corto plazo con prontitud.</t>
         </is>
       </c>
       <c r="M21" s="3" t="inlineStr">
@@ -2102,56 +2174,64 @@
       </c>
       <c r="N21" s="3" t="inlineStr">
         <is>
-          <t>Se espera que esta solición provisional de resultados mientras se adquieren los repuestos para reemplazar la pieza dañada (quebrada). Se sigiere remplazo a cotro plazo.</t>
+          <t>Se espera que la adquisición de los nuevos transductores ayude a garantizar la fiabilidad de los datos obtenidos en cada monitoreo fetal realizado con estos equipos.</t>
         </is>
       </c>
       <c r="O21" s="3" t="inlineStr">
         <is>
-          <t>La solcución es parcial ya que el fabricante Mindray descontinuó la linea y no vende el componenete dañado de forma individual. Se Logró encontrar la piea por medio de un vendedor particular y se planteó la cotizacion al gerente de mantenimiento para la adquixcicion de 2 sheaths ya que la del equipo de sala b muestra indicios del mismo tipo de desgaste. y la solucion del monitor de sala de hosp. A es temporal.</t>
+          <t>Los equipos actualmente se encuentran operacionales pero ante este tipo de desgaste el manual de servicio recomienda el reemplazo de los transductores para evitar errores en los estudios.</t>
         </is>
       </c>
       <c r="P21" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q21" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="Q21" s="3" t="n">
-        <v>2</v>
-      </c>
       <c r="R21" s="3" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>10:15</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>UCI A</t>
+          <t>Emergencia</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Cama quírurgica</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr"/>
+          <t>Balanzas Pediátricas y de adulto</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Detecto</t>
+        </is>
+      </c>
       <c r="H22" s="2" t="inlineStr"/>
-      <c r="I22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>127566</t>
+        </is>
+      </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
           <t>Correctivo</t>
@@ -2159,12 +2239,12 @@
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>La cama Hillrom P1900 fúe llevada al área de mantenimiento el por parte del personal de enfermeria ya que no realizaba los movieintos correspondientes de arriba y abajo unicamente levanta pierna y respladar. Se identifíco que el fluido hidráulico no estaba en su nivel. indicado por fabricante y ya requeria cambio.</t>
+          <t>Las balanzas pediátricas de emergencia se encontraron descalibradas en el recorrido matutino diario de las áreas, esto ya que fueron movidas y se descalibró el contrapeso.</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>Se realizo purgado del fluido hidráulico operando el dispositivo en todos sus movimientos para asegurar la salida de todo el fluido al recipiente del mismo. Se reemplazó por fluido nuevo y se coloco 1/4 de galón de fluido tal como lo exponse el manual de servicio del fabricante. Se opera todos los movimientos hidráulicos para asegurar el ingreso del fluido en todo el sistema. la cama queda funcional y operacional-</t>
+          <t>Se ajusto el tornillo del contrapeso cuidadosamente girando levemente a favor de las manecillas del reloj, soltando el indicador asegurando encontrara su punto de balance enmedio de la guia de peso.</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
@@ -2174,115 +2254,131 @@
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>Ya de regreso a su área se espera que el equipo sirva para los cuidados de pacientes en UCI. y se mantenda funcional hasta octubre cuando se tiene programado su mantenimiento preventivo.</t>
+          <t>Las personas ingresadas por medio de emergencias tendrán lecturas mas certeras de su peso lo cual es de mucha importancia para el personal de la salud al momento de suministrar medicamentos o determinar diagnósticos.</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr"/>
       <c r="P22" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q22" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="Q22" s="2" t="n">
-        <v>2</v>
-      </c>
       <c r="R22" s="2" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Quirófano 1</t>
+          <t>Laboratorio</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>Lámpara cielítica</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr"/>
-      <c r="H23" s="3" t="inlineStr"/>
-      <c r="I23" s="3" t="inlineStr"/>
+          <t>Centrífuga</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Drucker</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>755 VES</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>160960AB218</t>
+        </is>
+      </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>Correctivo</t>
+          <t>Revisión y Diagnóstico</t>
         </is>
       </c>
       <c r="K23" s="3" t="inlineStr">
         <is>
-          <t>Se solicitó revision y diagnósito por parte de mantenimineto ya que la lámapara cielitica de Q1, ya que no realizaba los movimientos correspondidnetes de las celdas LED al girar el mango rotatorio. Se identiíficoó que el mango salío del eje de soporte por movimientos de uso bruzco y soportes flojos.</t>
+          <t>Laboratorio solicitó revisión y diagnóstico de la centrífuga Drucker Horizon 755 VES. ya que esta no iniciaba y según relato del Dr. encargado del área (Rubén Vallecillo) emitió humo antes de dejar de funcionar. Se observó internamente una falla crítica en la tarjeta electrónica principal. Múltiples de los integrados de la placa presentan carbonización lo que compromete el funcionamiento del equipo.</t>
         </is>
       </c>
       <c r="L23" s="3" t="inlineStr">
         <is>
-          <t>Se logró colocar el mango rotatorio desplomado nuevamente en su eje ajustando todos los soportes y colocando una cantidad moderada de pegamentro de tornillos en el tornillo del eje que se inserta en el mango rotatorio. Se realizaron todas las pruebas de movimiento de las celdas LED con el mango rotatorio y realíza los movimientos. Se recomienda usar fuerza moderada al rotar o sujetar del mango.</t>
+          <t xml:space="preserve">La sustitución de los componentes microsoldados no resulta viable, ya que se corre el riesgo de comprometer otros componentes en el proceso. El equipo queda fuera de servicio hasta el reemplazo de la tarjeta principal. Se adjuntará cotización de la parte PN-7717041 (Placa electrónica principal centrífuga Drucker  Horizon 755 VES) al reporte entregado a mantenimiento para agilizar la respectiva compra / adquisición. Mientras tanto, el equipo queda de baja. Se recomienda una UPS de 1.5 KVA para mitigar el impacto de los picos de voltaje ya que la laca es inverter y susceptible a esto. </t>
         </is>
       </c>
       <c r="M23" s="3" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="N23" s="3" t="inlineStr">
         <is>
-          <t>Se espera que Q1 retome sus labores de cardiocirujía al día siguiente con la certeza que la lámpara cielitica cumpla su función de aportar iluminación al procedimiento y libertad de movimiento al personal de quirófano.</t>
-        </is>
-      </c>
-      <c r="O23" s="3" t="inlineStr"/>
+          <t>Se espera que por medio del reporte entregado a mantenimiento se pueda adquirir la placa para el reemplazo de la tarjeta su reparo, pruebas de funcionamiento y calibración para devolverlo en estado funcional y operable a su área (laboratorio)</t>
+        </is>
+      </c>
+      <c r="O23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El equipo queda fuera de servicio. El problema será recurrente ante la falta de un UPS para proteger el equipo de picos de voltaje. </t>
+        </is>
+      </c>
       <c r="P23" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q23" s="3" t="n">
         <v>1</v>
       </c>
       <c r="R23" s="3" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Quirófano 1</t>
+          <t>Laboratorio</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Intercambiador de temperatura quirírgico</t>
+          <t>Incubadora de Laboratorio</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr"/>
@@ -2295,12 +2391,12 @@
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>Se solicitó revisión y diagnóstico por parte de mantenimiento. Ya que el persnal reportó que el equipo "No enciende" por medio de una insepcción visual se determinó que fisicamente el equipo se ve en buen estado, una revisión detallada a sus partes destacó que la clavija y base del cable de alimentacíón estaban flijos, lo que no permitia contacto del cable con las clavijas L1, L2 Y N.</t>
+          <t>Se solicitò asistencia de parte de mantenimiento en el arèa de laboratorio ya qye su incubadora proncipal tiene emn mal estado la puerta, lo que pone en riesgo los cultivos dentro del mismo. Al examinar el equipo estaba unicamente cerrado con cinta adhesiva ya que el mecanismo de cierre se descompuso. Se desmontó la puerta para ver el mecanismo y se encuentra roto</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>Se desarmó el el enchufe del cable de alimentación para ajustar nuevamente L1, L2 y N, se cerró ajustando bien los tornillos de la base y se conectó fornfirmando correcto funcionamiento por 10 minutos. El equipo quedó en buen estado y funcional. Se sugiere no halar los cables al desconectar de la toma de pared.</t>
+          <t>Se soldó el seguro interno (Abrir/cerrar) de la puerta sujeto a la maniblea y se reemplazaron los tornillos por unos de mayor alcance para asegurar que no se salgan se sus ubicaciones.</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
@@ -2310,7 +2406,7 @@
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>Se espera opere correctamente al dia siguiente duarnte la cirugia de corazón abierto al calnetar la sangre del paciente mientras esta se encuentra en estado extracorpóreo para evitar choques térmicos y poner en riesgo al peciante.</t>
+          <t>Se esper que el personal siga las recomendaciones de no ejercer fuerza excesiva al abrir y cerrar ya que el mecanismo puede volver a quebrarse.</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr"/>
@@ -2318,9 +2414,489 @@
         <v>1</v>
       </c>
       <c r="Q24" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="R24" s="2" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="n">
+        <v>61</v>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>UCIN</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Incubadora Neonatal</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr"/>
+      <c r="H25" s="3" t="inlineStr"/>
+      <c r="I25" s="3" t="inlineStr"/>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>Correctivo</t>
+        </is>
+      </c>
+      <c r="K25" s="3" t="inlineStr">
+        <is>
+          <t>La Incubadora noenatal GE giraffe Omnibed presenta probelmas perisistentes en su motor. Anteriormente se realizó antenimimento correctivo de las balineras. Actuakmente se solicita ayuda por "Sonidos fuertes" provinientes del dispositivo.</t>
+        </is>
+      </c>
+      <c r="L25" s="3" t="inlineStr">
+        <is>
+          <t>Posterior al analisis de los componentes internos una ves se remueve su carcaza, se determino que piezas especificas como el motor, sensor optico, plasticos de acoplo requieren ser reemplazados,</t>
+        </is>
+      </c>
+      <c r="M25" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N25" s="3" t="inlineStr">
+        <is>
+          <t>Se esperan solicitudoes de atencion por el sonido intermitente que recurre en el motor. Se solci´to la compra de respuestos para atender el problema de raiz.</t>
+        </is>
+      </c>
+      <c r="O25" s="3" t="inlineStr">
+        <is>
+          <t>queda operacional con los ruidos intermitentes.y se recomienda el reemplazo de las piezas entregadas a gerente de mantenimineto con sus repspectiva cotización para compra.</t>
+        </is>
+      </c>
+      <c r="P25" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="R24" s="2" t="n">
+      <c r="Q25" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="R25" s="3" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>9:00</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Tomgrafo</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Correctivo</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Se hizó al la observación al peronal de Biotec que el inicializar el tomógrafo CT-300 Philips en cada báarido aparecia un mensaje de error emitido por el software. Tras una revisión de determino que el disco duro estaba próximo a alacanzar su capacidad máximo la que pone en riesgo la "Raw data" ante corrupciones por sobre carga de información, de igual forma se expuso que el equipo se mantiene encendido 24/7.</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>Se recomendó al personal depurar de estudios muy antiguos el disco duro del ordenador. Ya que la sobrecarga del mismo presenta el riesgo de coorromper la raw data de estudios recientes. El sistema muestra advenrtencias por esta situación, pero ningun error fatal de sistema si se siguen las indicaciones. De igual forma se recomendó apagar el ordenador un par de minutos mínimo 1 vezpor semana.</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>Se espera que el persnal siga las recomiendaciones e indicaciones del personal técncico para evitar la sobre carga del disco duro, ya que esto pone en riesgo la calidad de los estudios y la información adquirida para diagnóstico.</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr"/>
+      <c r="P26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q26" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="R26" s="2" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="n">
+        <v>63</v>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Hospitalización A</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>Termómetro de oído</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr"/>
+      <c r="H27" s="3" t="inlineStr"/>
+      <c r="I27" s="3" t="inlineStr"/>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>Correctivo</t>
+        </is>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>En una visita al área, personal de enfermería de Hospitalización B expusó que los termometro de oido portátil del MSV Welch Allyn LXI 45NTO Tenia sus baterías descargadas. Se canbiaron las mismas por unas cagadas y el termómetro no operó. Al ver sus componentes internos, se observía que en su placa un falso contacto con la bandeja de batería por el desgaste de la constante driccion entre la bandeja y la placa.</t>
+        </is>
+      </c>
+      <c r="L27" s="3" t="inlineStr">
+        <is>
+          <t>Posterior a la vista intenra de la tarjeta del equipo se realizaron varias pruebas de utilizando aluminio como medio de conduccion entre la placa y la bandeja de bateria. Estas pruebas no dieron resultado ya que el plastico de cierre ya estaba sumamente desgastado lo que no permitia que cerrara bien. Como existe repuesto total del dispositovo se optó por remplazarlo en su totalidad. y queda funcional y operando.</t>
+        </is>
+      </c>
+      <c r="M27" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="N27" s="3" t="inlineStr">
+        <is>
+          <t>Al ser equipo de atiguedad dentro del área, se sepera que termomentro adjunto al MSV de su vida util para reemplazar el monitor en su totalidad.</t>
+        </is>
+      </c>
+      <c r="O27" s="3" t="inlineStr"/>
+      <c r="P27" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q27" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="R27" s="3" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Hospitalización B</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Monitor de Signos vitales</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>Correctivo</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Se solicitó apoyo de por medio de un aorden de mantenimiento para inspeccionar el MSV Mindray VS-900 C de Hospitalización A, ya que este no sensa temperatura y la sonda de temperatura parece estar en buen estado. Se inpseccionó mas a detalle internamente y se determinó que el "sheath" o funda donde se coloca la sonda de temp. esta rota. y la guia de la misma no hace contacto con el sensor por medio de una botornera.</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>Se implemento el ingenio para elaborar una extensión a la funda que hace contacto con el sensor ya que este fue el que se quebró e impide el funcionamiento del módulo de temperatura del MSV. Se lógro proporcionar esta solución temporal y el equipo queda funacional tras varias pruebas.</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>Se espera que esta solición provisional de resultados mientras se adquieren los repuestos para reemplazar la pieza dañada (quebrada). Se sigiere remplazo a cotro plazo.</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>La solcución es parcial ya que el fabricante Mindray descontinuó la linea y no vende el componenete dañado de forma individual. Se Logró encontrar la piea por medio de un vendedor particular y se planteó la cotizacion al gerente de mantenimiento para la adquixcicion de 2 sheaths ya que la del equipo de sala b muestra indicios del mismo tipo de desgaste. y la solucion del monitor de sala de hosp. A es temporal.</t>
+        </is>
+      </c>
+      <c r="P28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q28" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="R28" s="2" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="n">
+        <v>65</v>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>UCI A</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>Cama quírurgica</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr"/>
+      <c r="H29" s="3" t="inlineStr"/>
+      <c r="I29" s="3" t="inlineStr"/>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>Correctivo</t>
+        </is>
+      </c>
+      <c r="K29" s="3" t="inlineStr">
+        <is>
+          <t>La cama Hillrom P1900 fúe llevada al área de mantenimiento el por parte del personal de enfermeria ya que no realizaba los movieintos correspondientes de arriba y abajo unicamente levanta pierna y respladar. Se identifíco que el fluido hidráulico no estaba en su nivel. indicado por fabricante y ya requeria cambio.</t>
+        </is>
+      </c>
+      <c r="L29" s="3" t="inlineStr">
+        <is>
+          <t>Se realizo purgado del fluido hidráulico operando el dispositivo en todos sus movimientos para asegurar la salida de todo el fluido al recipiente del mismo. Se reemplazó por fluido nuevo y se coloco 1/4 de galón de fluido tal como lo exponse el manual de servicio del fabricante. Se opera todos los movimientos hidráulicos para asegurar el ingreso del fluido en todo el sistema. la cama queda funcional y operacional-</t>
+        </is>
+      </c>
+      <c r="M29" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="N29" s="3" t="inlineStr">
+        <is>
+          <t>Ya de regreso a su área se espera que el equipo sirva para los cuidados de pacientes en UCI. y se mantenda funcional hasta octubre cuando se tiene programado su mantenimiento preventivo.</t>
+        </is>
+      </c>
+      <c r="O29" s="3" t="inlineStr"/>
+      <c r="P29" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q29" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="R29" s="3" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Quirófano 1</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Lámpara cielítica</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr"/>
+      <c r="H30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="inlineStr"/>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>Correctivo</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Se solicitó revision y diagnósito por parte de mantenimineto ya que la lámapara cielitica de Q1, ya que no realizaba los movimientos correspondidnetes de las celdas LED al girar el mango rotatorio. Se identiíficoó que el mango salío del eje de soporte por movimientos de uso bruzco y soportes flojos.</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>Se logró colocar el mango rotatorio desplomado nuevamente en su eje ajustando todos los soportes y colocando una cantidad moderada de pegamentro de tornillos en el tornillo del eje que se inserta en el mango rotatorio. Se realizaron todas las pruebas de movimiento de las celdas LED con el mango rotatorio y realíza los movimientos. Se recomienda usar fuerza moderada al rotar o sujetar del mango.</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>Se espera que Q1 retome sus labores de cardiocirujía al día siguiente con la certeza que la lámpara cielitica cumpla su función de aportar iluminación al procedimiento y libertad de movimiento al personal de quirófano.</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="inlineStr"/>
+      <c r="P30" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q30" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R30" s="2" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="n">
+        <v>67</v>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Quirófano 1</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>Intercambiador de temperatura quirírgico</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr"/>
+      <c r="H31" s="3" t="inlineStr"/>
+      <c r="I31" s="3" t="inlineStr"/>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>Correctivo</t>
+        </is>
+      </c>
+      <c r="K31" s="3" t="inlineStr">
+        <is>
+          <t>Se solicitó revisión y diagnóstico por parte de mantenimiento. Ya que el persnal reportó que el equipo "No enciende" por medio de una insepcción visual se determinó que fisicamente el equipo se ve en buen estado, una revisión detallada a sus partes destacó que la clavija y base del cable de alimentacíón estaban flijos, lo que no permitia contacto del cable con las clavijas L1, L2 Y N.</t>
+        </is>
+      </c>
+      <c r="L31" s="3" t="inlineStr">
+        <is>
+          <t>Se desarmó el el enchufe del cable de alimentación para ajustar nuevamente L1, L2 y N, se cerró ajustando bien los tornillos de la base y se conectó fornfirmando correcto funcionamiento por 10 minutos. El equipo quedó en buen estado y funcional. Se sugiere no halar los cables al desconectar de la toma de pared.</t>
+        </is>
+      </c>
+      <c r="M31" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="N31" s="3" t="inlineStr">
+        <is>
+          <t>Se espera opere correctamente al dia siguiente duarnte la cirugia de corazón abierto al calnetar la sangre del paciente mientras esta se encuentra en estado extracorpóreo para evitar choques térmicos y poner en riesgo al peciante.</t>
+        </is>
+      </c>
+      <c r="O31" s="3" t="inlineStr"/>
+      <c r="P31" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q31" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="R31" s="3" t="n">
         <v>30</v>
       </c>
     </row>

</xml_diff>